<commit_message>
refactor: restrict agent tool access by removing doc search tools and update graph node source locations
</commit_message>
<xml_diff>
--- a/ap_citizen360_v2.0/database/query_log.xlsx
+++ b/ap_citizen360_v2.0/database/query_log.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K45"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2243,7 +2243,6 @@
           <t>Count is 10</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
       <c r="I45" t="n">
         <v>2.1</v>
       </c>
@@ -2252,6 +2251,481 @@
       </c>
       <c r="K45" t="n">
         <v>2.5</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-08-09 23:15:46</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>test_user</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>386a61ce-cee6-4689-9de1-c462a3f02148</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>hi</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Hello, test_user! I am the **Citizen360 AI Assistant**, your intelligent data and document assistant for the AP Citizen360 platform.
+How can I help you today? You can ask me about:
+- Student dropout risk lists and school performance hotspots
+- Teacher attendance and academic marks analysis
+- Welfare scheme delivery gaps and eligibility criteria
+- Policy documents, circulars, and official guidelines</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Hello, test_user! I am the **Citizen360 AI Assistant**, your intelligent data and document assistant for the AP Citizen360 platform.
+How can I help you today? You can ask me about:
+- Student dropout risk lists and school performance hotspots
+- Teacher attendance and academic marks analysis
+- Welfare scheme delivery gaps and eligibility criteria
+- Policy documents, circulars, and official guidelines</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-08-09 23:16:46</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>test_user</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>386a61ce-cee6-4689-9de1-c462a3f02148</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>"Give me class 6 students in &lt;PERSON&gt; who dropped out in 2025-26."</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Hello, test_user! I am the **Citizen360 AI Assistant**, your intelligent data and document assistant for the AP Citizen360 platform.
+How can I help you today? You can ask me about:
+- Student dropout risk lists and school performance hotspots
+- Teacher attendance and academic marks analysis
+- Welfare scheme delivery gaps and eligibility criteria
+- Policy documents, circulars, and official guidelines</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Hello, test_user! I am the **Citizen360 AI Assistant**, your intelligent data and document assistant for the AP Citizen360 platform.
+How can I help you today? You can ask me about:
+- Student dropout risk lists and school performance hotspots
+- Teacher attendance and academic marks analysis
+- Welfare scheme delivery gaps and eligibility criteria
+- Policy documents, circulars, and official guidelines</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" t="n">
+        <v>12.19</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-08-09 23:17:11</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>test_user</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>386a61ce-cee6-4689-9de1-c462a3f02148</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Give me class 6 students in &lt;PERSON&gt; who dropped out in 2025-26.</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Hello, test_user! I am the **Citizen360 AI Assistant**, your intelligent data and document assistant for the AP Citizen360 platform.
+How can I help you today? You can ask me about:
+- Student dropout risk lists and school performance hotspots
+- Teacher attendance and academic marks analysis
+- Welfare scheme delivery gaps and eligibility criteria
+- Policy documents, circulars, and official guidelines</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Hello, test_user! I am the **Citizen360 AI Assistant**, your intelligent data and document assistant for the AP Citizen360 platform.
+How can I help you today? You can ask me about:
+- Student dropout risk lists and school performance hotspots
+- Teacher attendance and academic marks analysis
+- Welfare scheme delivery gaps and eligibility criteria
+- Policy documents, circulars, and official guidelines</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" t="n">
+        <v>3.03</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-08-09 23:33:14</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>test_user</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>386a61ce-cee6-4689-9de1-c462a3f02148</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Give me class 6 students in anantapuramu who dropped out in 2025-26.</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>I do not have access to any document passages, circulars, or guidelines that discuss the education of Class 6 students in Anantapuramu who dropped out in 2025-26. Without the specific document or circulars you are referring to, I cannot answer your question based on the available information.</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>I do not have access to any document passages, circulars, or guidelines that discuss the education of Class 6 students in Anantapuramu who dropped out in 2025-26. Without the specific document or circulars you are referring to, I cannot answer your question based on the available information.</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>0</v>
+      </c>
+      <c r="J49" t="n">
+        <v>12.02</v>
+      </c>
+      <c r="K49" t="n">
+        <v>23.77</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-08-09 23:41:27</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>test_user</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>386a61ce-cee6-4689-9de1-c462a3f02148</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Give me class 6 students in anantapuramu who dropped out in 2025-26.</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>!
+&lt;tool_call&gt;
+&lt;function=execute_sql&gt;
+&lt;parameter=query&gt;
+SELECT * FROM citizen_student WHERE district_name = 'Anantapuramu' AND academic_year = '2025-26' AND current_grade = '6'
+&lt;/parameter&gt;
+&lt;/function&gt;
+&lt;/tool_call&gt;</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>!
+&lt;tool_call&gt;
+&lt;function=execute_sql&gt;
+&lt;parameter=query&gt;
+SELECT * FROM citizen_student WHERE district_name = 'Anantapuramu' AND academic_year = '2025-26' AND current_grade = '6'
+&lt;/parameter&gt;
+&lt;/function&gt;
+&lt;/tool_call&gt;</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="J50" t="n">
+        <v>0</v>
+      </c>
+      <c r="K50" t="n">
+        <v>9.81</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-08-09 23:44:14</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>test_user</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>386a61ce-cee6-4689-9de1-c462a3f02148</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Give me class 6 students in anantapuramu who dropped out in 2025-26.</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Based on the context, I am the **Citizen360 AI Assistant**, your intelligent data and document assistant for the AP Citizen360 platform.
+How can I help you today? You can ask me about:
+- Student dropout risk lists and school performance hotspots
+- Teacher attendance and academic marks analysis
+- Welfare scheme delivery gaps and eligibility criteria
+- Policy documents, circulars, and official guidelines</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Based on the context, I am the **Citizen360 AI Assistant**, your intelligent data and document assistant for the AP Citizen360 platform.
+How can I help you today? You can ask me about:
+- Student dropout risk lists and school performance hotspots
+- Teacher attendance and academic marks analysis
+- Welfare scheme delivery gaps and eligibility criteria
+- Policy documents, circulars, and official guidelines</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="J51" t="n">
+        <v>0</v>
+      </c>
+      <c r="K51" t="n">
+        <v>13.05</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-08-09 23:51:41</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>test_user</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>f1d418c1-3fe3-4df3-8ab7-6259754f8880</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Give me class 6 students in anantapuramu who dropped out in 2025-26.</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>-- Model failed to emit tool. Force retry for: Give me class 6 students in anantapuramu who dropped out in 2025-26.</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>SQL execution failed: Only SELECT statements are allowed</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Only SELECT statements are allowed</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>65.52</v>
+      </c>
+      <c r="J52" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="K52" t="n">
+        <v>80.28</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-08-09 23:56:24</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>test_user</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>784d1803-01ca-4185-b140-09bad573210d</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Give me class 6 students in anantapuramu who dropped out in 2025-26.</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>-- Model failed to emit tool. Force retry for: Give me class 6 students in anantapuramu who dropped out in 2025-26.</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>SQL execution failed: Only SELECT statements are allowed</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Only SELECT statements are allowed</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>102.46</v>
+      </c>
+      <c r="J53" t="n">
+        <v>4.17</v>
+      </c>
+      <c r="K53" t="n">
+        <v>118.28</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-08-09 23:59:33</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>test_user</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>254e605e-6a64-446d-b021-8a696a609eca</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Give me class 6 students in anantapuramu who dropped out in 2025-26.</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>cancelled</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Request cancelled by user.</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" t="n">
+        <v>0</v>
+      </c>
+      <c r="K54" t="n">
+        <v>86.34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>